<commit_message>
feat: converted .xlsx files to pdf for vertex ai chunking
</commit_message>
<xml_diff>
--- a/public/docs/pdf-md-pdf/complete data of Kattakada (1)/block panchayat divisions.xlsx
+++ b/public/docs/pdf-md-pdf/complete data of Kattakada (1)/block panchayat divisions.xlsx
@@ -397,25 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:C22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Name</v>
       </c>
       <c r="B1" t="str">
-        <v/>
+        <v>BP_DIVISION</v>
       </c>
       <c r="C1" t="str">
-        <v>BP_DIVISION</v>
-      </c>
-      <c r="D1" t="str">
-        <v/>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
         <v>BP_MEMBER</v>
       </c>
     </row>
@@ -424,18 +415,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>10 - Killi / 06 - Vellanad</v>
       </c>
       <c r="C2" t="str">
-        <v>10 - Killi / 06 - Vellanad</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
         <v>Sreekutty Sathish</v>
       </c>
     </row>
@@ -444,18 +426,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C3" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -464,18 +437,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C4" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
         <v>Sarala</v>
       </c>
     </row>
@@ -484,18 +448,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>10 - Killi / 06 - Vellanad</v>
       </c>
       <c r="C5" t="str">
-        <v>10 - Killi / 06 - Vellanad</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
         <v>Sreekutty Sathish</v>
       </c>
     </row>
@@ -504,18 +459,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C6" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
         <v>Sarala</v>
       </c>
     </row>
@@ -524,18 +470,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C7" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
         <v>Sarala</v>
       </c>
     </row>
@@ -544,18 +481,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C8" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
         <v>Sarala</v>
       </c>
     </row>
@@ -564,18 +492,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B9" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C9" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
         <v>Sarala</v>
       </c>
     </row>
@@ -584,18 +503,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C10" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
         <v>Sarala</v>
       </c>
     </row>
@@ -604,18 +514,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C11" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -624,18 +525,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B12" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C12" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -644,18 +536,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C13" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -664,18 +547,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B14" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C14" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -684,18 +558,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B15" t="str">
-        <v/>
+        <v>10 - Killi / 06 - Vellanad</v>
       </c>
       <c r="C15" t="str">
-        <v>10 - Killi / 06 - Vellanad</v>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-      <c r="F15" t="str">
         <v>Sreekutty Sathish</v>
       </c>
     </row>
@@ -704,18 +569,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B16" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C16" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
         <v>Sarala</v>
       </c>
     </row>
@@ -724,18 +580,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>10 - Killi / 06 - Vellanad</v>
       </c>
       <c r="C17" t="str">
-        <v>10 - Killi / 06 - Vellanad</v>
-      </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
         <v>Sreekutty Sathish</v>
       </c>
     </row>
@@ -744,18 +591,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>10 - Killi / 06 - Vellanad</v>
       </c>
       <c r="C18" t="str">
-        <v>10 - Killi / 06 - Vellanad</v>
-      </c>
-      <c r="D18" t="str">
-        <v/>
-      </c>
-      <c r="E18" t="str">
-        <v/>
-      </c>
-      <c r="F18" t="str">
         <v>Sreekutty Sathish</v>
       </c>
     </row>
@@ -764,18 +602,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C19" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D19" t="str">
-        <v/>
-      </c>
-      <c r="E19" t="str">
-        <v/>
-      </c>
-      <c r="F19" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -784,18 +613,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C20" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D20" t="str">
-        <v/>
-      </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -804,18 +624,9 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>09 - Kattakada / 06 - Vellanad</v>
       </c>
       <c r="C21" t="str">
-        <v>09 - Kattakada / 06 - Vellanad</v>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
-      <c r="E21" t="str">
-        <v/>
-      </c>
-      <c r="F21" t="str">
         <v>Sunitha V.J</v>
       </c>
     </row>
@@ -824,24 +635,15 @@
         <v>32 - Kattakada</v>
       </c>
       <c r="B22" t="str">
-        <v/>
+        <v>08 - Amachel / 06 - Vellanad</v>
       </c>
       <c r="C22" t="str">
-        <v>08 - Amachel / 06 - Vellanad</v>
-      </c>
-      <c r="D22" t="str">
-        <v/>
-      </c>
-      <c r="E22" t="str">
-        <v/>
-      </c>
-      <c r="F22" t="str">
         <v>Sarala</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>